<commit_message>
Fix: replace all xlsx formulas with literal values
openpyxl clears cached formula values (<v/>) on save, so cells like
C43 (=C9) exported as <f>C9</f><v /> — empty. SheetJS read null for
every model URL and no GLB loaded.

Replaced all 15 formula cells (=C9, =C13, =C11 etc. across scenes
0-5) with their resolved literal values (the actual https:// URLs).
This makes the xlsx self-contained: no formula evaluation needed,
SheetJS reads the URL strings directly.
</commit_message>
<xml_diff>
--- a/demo2-xlsx/demo2-input_3.xlsx
+++ b/demo2-xlsx/demo2-input_3.xlsx
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:O717"/>
+  <dimension ref="A1:O717"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="72" min="1" max="1"/>
@@ -2932,13 +2932,15 @@
       <c r="A43" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="B43" s="9">
-        <f>B9</f>
-        <v/>
-      </c>
-      <c r="C43" s="29">
-        <f>C9</f>
-        <v/>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>City Model v2</t>
+        </is>
+      </c>
+      <c r="C43" s="29" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2city-opt-v2.glb</t>
+        </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
@@ -2987,13 +2989,15 @@
       <c r="A44" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="B44" s="14">
-        <f>B13</f>
-        <v/>
-      </c>
-      <c r="C44" s="31">
-        <f>C13</f>
-        <v/>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Kopuk Normal Facade v5</t>
+        </is>
+      </c>
+      <c r="C44" s="31" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2kopuk-normalfacade-opt-v5.glb</t>
+        </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
@@ -6732,9 +6736,10 @@
           <t>City Model v2 (S0'dan devralınır)</t>
         </is>
       </c>
-      <c r="C115" s="53">
-        <f>C9</f>
-        <v/>
+      <c r="C115" s="53" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2city-opt-v2.glb</t>
+        </is>
       </c>
       <c r="D115" s="11" t="inlineStr">
         <is>
@@ -6788,9 +6793,10 @@
           <t>Kopuk Normal Facade v5 (S0'dan devralınır)</t>
         </is>
       </c>
-      <c r="C116" s="54">
-        <f>C13</f>
-        <v/>
+      <c r="C116" s="54" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2kopuk-normalfacade-opt-v5.glb</t>
+        </is>
       </c>
       <c r="D116" s="16" t="inlineStr">
         <is>
@@ -7605,6 +7611,7 @@
         </is>
       </c>
     </row>
+    <row r="127"/>
     <row r="128" ht="9.75" customHeight="1" s="72"/>
     <row r="129" ht="21.75" customHeight="1" s="72">
       <c r="A129" s="80" t="inlineStr">
@@ -14160,9 +14167,10 @@
           <t>City Model v2</t>
         </is>
       </c>
-      <c r="C250" s="63">
-        <f>C9</f>
-        <v/>
+      <c r="C250" s="63" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2city-opt-v2.glb</t>
+        </is>
       </c>
       <c r="D250" s="11" t="inlineStr">
         <is>
@@ -14216,9 +14224,10 @@
           <t>City White Facade v3</t>
         </is>
       </c>
-      <c r="C251" s="53">
-        <f>C12</f>
-        <v/>
+      <c r="C251" s="53" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2city-whitefacade-v3.glb</t>
+        </is>
       </c>
       <c r="D251" s="11" t="inlineStr">
         <is>
@@ -14272,9 +14281,10 @@
           <t>City Metal v1</t>
         </is>
       </c>
-      <c r="C252" s="53">
-        <f>C11</f>
-        <v/>
+      <c r="C252" s="53" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2city-metal-v1.glb</t>
+        </is>
       </c>
       <c r="D252" s="11" t="inlineStr">
         <is>
@@ -14328,9 +14338,10 @@
           <t>Kopuk Normal Facade v5</t>
         </is>
       </c>
-      <c r="C253" s="54">
-        <f>C13</f>
-        <v/>
+      <c r="C253" s="54" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2kopuk-normalfacade-opt-v5.glb</t>
+        </is>
       </c>
       <c r="D253" s="16" t="inlineStr">
         <is>
@@ -19895,9 +19906,10 @@
           <t>City Metal v1</t>
         </is>
       </c>
-      <c r="C356" s="53">
-        <f>C11</f>
-        <v/>
+      <c r="C356" s="53" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2city-metal-v1.glb</t>
+        </is>
       </c>
       <c r="D356" s="11" t="inlineStr">
         <is>
@@ -19951,9 +19963,10 @@
           <t>Sehiriçi Apartman v6</t>
         </is>
       </c>
-      <c r="C357" s="54">
-        <f>C14</f>
-        <v/>
+      <c r="C357" s="54" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2-sehirici-apartmanici-opt-v6.glb</t>
+        </is>
       </c>
       <c r="D357" s="16" t="inlineStr">
         <is>
@@ -23696,9 +23709,10 @@
           <t>Interior Apartment v4</t>
         </is>
       </c>
-      <c r="C427" s="54">
-        <f>C15</f>
-        <v/>
+      <c r="C427" s="54" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2interior-soloapartement-opt-v4.glb</t>
+        </is>
       </c>
       <c r="D427" s="16" t="inlineStr">
         <is>
@@ -36463,9 +36477,10 @@
           <t>Interior Apartment v4</t>
         </is>
       </c>
-      <c r="C654" s="53">
-        <f>C15</f>
-        <v/>
+      <c r="C654" s="53" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/DEMO2interior-soloapartement-opt-v4.glb</t>
+        </is>
       </c>
       <c r="D654" s="11" t="inlineStr">
         <is>
@@ -36519,9 +36534,10 @@
           <t>Scene 5 Collider</t>
         </is>
       </c>
-      <c r="C655" s="54">
-        <f>C16</f>
-        <v/>
+      <c r="C655" s="54" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/decentralize-dfw/vea-randomfiles/main/SCENE5-COLLDERd.glb</t>
+        </is>
       </c>
       <c r="D655" s="16" t="inlineStr">
         <is>

</xml_diff>